<commit_message>
reporta todo telefone descartado, nao so a celula 100% lixo
Conferindo o adapter contra a planilha REAL (nao a fixture), os totais nao
fechavam: 331 telefones e 3 linhas de lixo, mas so 2 rejeicoes reportadas. A
terceira (QUADRA 05 CHACARA 03/08) convive com um numero valido na mesma
celula — e era descartada em SILENCIO, exatamente o defeito que este
importador existe para nao repetir.

Passa a reportar sempre que houve descarte, distinguindo os dois casos:
"pessoa importada sem telefone" (celula toda lixo) e "N descartado(s), os M
validos foram importados".

Fixture ganhou o caso correspondente (GINA: telefone bom + lixo na mesma
celula) e o teste que prova o relato.

Leitura da planilha real: 242 pessoas (229 proprietarios + 13 relacionadas),
229 unidades, 331 telefones, 3 rejeicoes — todas de telefone, nenhuma pessoa
perdida. Suite da frente 2938/2938.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/tests/Fixtures/Cobranca/importacao/cadastro_condominos_amostra.xlsx
+++ b/app/tests/Fixtures/Cobranca/importacao/cadastro_condominos_amostra.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="59">
   <si>
     <t>CONTABIL EXEMPLO LTDA</t>
   </si>
@@ -171,13 +171,29 @@
     <t>666.777.888-23</t>
   </si>
   <si>
+    <t>Emissão: 29/07/2026 16:08</t>
+  </si>
+  <si>
+    <t>CONTABIL EXEMPLO LTDA - Rua Exemplo, 1</t>
+  </si>
+  <si>
     <t>Filtros: Unidades: Todas</t>
   </si>
   <si>
-    <t>CONTABIL EXEMPLO LTDA - Rua Exemplo, 1</t>
-  </si>
-  <si>
-    <t>Emissão: 29/07/2026 16:08</t>
+    <t>QUADRA 01 CHACARA 01/07</t>
+  </si>
+  <si>
+    <t>GINA EXEMPLO CASTRO</t>
+  </si>
+  <si>
+    <t>777.888.999-34</t>
+  </si>
+  <si>
+    <t>Área Rural - S/N - QUADRA 01 CHACARA 01/07 - LAGO EXEMPLO - Cidade Exemplo - GO - CEP: 72900-000</t>
+  </si>
+  <si>
+    <t>+55 (61) 900000007
+null () null</t>
   </si>
 </sst>
 </file>
@@ -517,7 +533,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -525,25 +541,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:8"/>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8"/>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:8"/>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:8"/>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>4</v>
@@ -742,20 +754,43 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:8"/>
-    <row r="19" spans="1:8">
-      <c r="A19" t="s">
-        <v>51</v>
-      </c>
-    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" t="s">
+        <v>57</v>
+      </c>
+      <c r="H18" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8"/>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>53</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>